<commit_message>
docs(reports): deploy unified consolidated summary reports for build 19
</commit_message>
<xml_diff>
--- a/reports/history/android/build-19/Excel/Failed_Test_Cases.xlsx
+++ b/reports/history/android/build-19/Excel/Failed_Test_Cases.xlsx
@@ -482,12 +482,12 @@
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="9620" customWidth="1" min="8" max="8"/>
+    <col width="9433" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="40" customHeight="1">
@@ -543,7 +543,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>TC_GEN_008</t>
+          <t>TC_GEN_002</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>test_responsive_ui_smoke</t>
+          <t>test_auth_invalid_credentials</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -568,152 +568,132 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>26.96</t>
+          <t>27.76</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23 08:10:41</t>
+          <t>2026-06-24 01:32:38</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t>@pytest.fixture(scope="function")
-    def driver():
-        """Initializes and yields Appium driver targeting the debug APK."""
-        # Resolve APK path relative to conftest.py
-        base_dir = os.path.dirname(os.path.dirname(os.path.dirname(os.path.abspath(__file__))))
-        apk_path = os.path.join(base_dir, "build", "app", "outputs", "flutter-apk", "app-debug.apk")
-        options = UiAutomator2Options()
-        options.platform_name = "Android"
-        options.automation_name = "UiAutomator2"
-        options.device_name = "Android Emulator"
-        options.app = apk_path
-        options.no_reset = False
-        options.auto_grant_permissions = True
-        # Optional settings to allow file/camera access mock
-        options.set_capability("gpsEnabled", "true")
-        print(f"[MobileConftest] Launching Appium driver targeting: {apk_path}")
-&gt;       driver = webdriver.Remote(APPIUM_SERVER_URL, options=options)
-                 ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
-tests/mobile_e2e/conftest.py:32: 
+          <t>driver = &lt;appium.webdriver.webdriver.WebDriver (session="8df9b57d-e778-4b63-9dc7-3ab099e509dd")&gt;
+    def test_auth_invalid_credentials(driver):
+        """Test that login with invalid credentials displays an error on mobile."""
+        time.sleep(3)
+        login_page = LoginPage(driver)
+&gt;       login_page.login("nonexistent_farmer@kisan.com", "WrongPass123!")
+tests/mobile_e2e/test_suites/test_auth.py:25: 
 _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ 
-/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/appium/webdriver/webdriver.py:251: in __init__
-    super().__init__(
-/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/selenium/webdriver/remote/webdriver.py:300: in __init__
-    self.start_session(capabilities)
-/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/appium/webdriver/webdriver.py:345: in start_session
-    response = self.execute(RemoteCommand.NEW_SESSION, w3c_caps)
-               ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests/mobile_e2e/pages/login_page.py:14: in login
+    self.send_keys(self.EMAIL_INPUT, email)
+tests/mobile_e2e/pages/base_page.py:31: in send_keys
+    element = self.wait_for_element(locator)
+              ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+tests/mobile_e2e/pages/base_page.py:22: in wait_for_element
+    raise e
+tests/mobile_e2e/pages/base_page.py:17: in wait_for_element
+    return WebDriverWait(self.driver, self.timeout).until(
+/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/selenium/webdriver/support/wait.py:112: in until
+    value = method(self._driver)
+            ^^^^^^^^^^^^^^^^^^^^
+/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/selenium/webdriver/support/expected_conditions.py:188: in _predicate
+    return _element_if_visible(driver.find_element(*locator))
+                               ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
+/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/selenium/webdriver/remote/webdriver.py:899: in find_element
+    return self.execute(Command.FIND_ELEMENT, {"using": by, "value": value})["value"]
+           ^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^^
 /opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/selenium/webdriver/remote/webdriver.py:492: in execute
     self.error_handler.check_response(response)
 _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ _ 
-self = &lt;selenium.webdriver.remote.errorhandler.ErrorHandler object at 0x7f2b58a2c1d0&gt;
-response = {'status': 500, 'value': '{"value":{"error":"unknown error","message":"Cannot start the \'com.kisanmitra.kisan_mitra\'...e/node/20.20.2/x64/lib/node_modules/appium/node_modules/@appium/base-driver/build/lib/protocol/protocol.js:401:25)"}}'}
-    def check_response(self, response: dict[str, Any]) -&gt; None:
-        """Check that a JSON response from the WebDriver does not have an error.
-        Args:
-            response: The JSON response from the WebDriver server as a dictionary
-                object.
-        Raises:
-            WebDriverException: If the response contains an error message.
+self = &lt;appium.webdriver.errorhandler.MobileErrorHandler object at 0x7f2b9cc46990&gt;
+response = {'status': 500, 'value': '{"value":{"error":"unknown error","message":"io.appium.uiautomator2.common.exceptions.UiAuto...r2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath1(AccessibilityNodeInfoDumper.java:279)\\n\\t... 33 more\\n"}}'}
+    def check_response(self, response: Dict[str, Any]) -&gt; None:
         """
-        status = response.get("status", None)
-        if not status or status == ErrorCode.SUCCESS:
+        https://www.w3.org/TR/webdriver/#errors
+        """
+        payload = response.get('value', '')
+        if isinstance(payload, dict):
+            payload_dict = payload
+        else:
+            try:
+                payload_dict = json.loads(payload)
+            except (json.JSONDecodeError, TypeError):
+                return
+            if not isinstance(payload_dict, dict):
+                return
+        value = payload_dict.get('value')
+        if not isinstance(value, dict):
             return
-        value = None
-        message = response.get("message", "")
-        screen: str = response.get("screen", "")
-        stacktrace = None
-        if isinstance(status, int):
-            value_json = response.get("value", None)
-            if value_json and isinstance(value_json, str):
-                try:
-                    value = json.loads(value_json)
-                    if isinstance(value, dict):
-                        if len(value) == 1:
-                            value = value["value"]
-                        status = value.get("error", None)
-                        if not status:
-                            status = value.get("status", ErrorCode.UNKNOWN_ERROR)
-                            message = value.get("value") or value.get("message")
-                            if not isinstance(message, str):
-                                value = message
-                                message = message.get("message") if isinstance(message, dict) else None
-                        else:
-                            message = value.get("message", None)
-                except ValueError:
-                    pass
-        exception_class: type[WebDriverException]
-        e = ErrorCode()
-        error_codes = [item for item in dir(e) if not item.startswith("__")]
-        for error_code in error_codes:
-            error_info = getattr(ErrorCode, error_code)
-            if isinstance(error_info, list) and status in error_info:
-                exception_class = getattr(ExceptionMapping, error_code, WebDriverException)
-                break
-        else:
-            exception_class = WebDriverException
-        if not value:
-            value = response["value"]
-        if isinstance(value, str):
-            raise exception_class(value)
-        if message == "" and "message" in value:
-            message = value["message"]
-        screen = None  # type: ignore[assignment]
-        if "screen" in value:
-            screen = value["screen"]
-        stacktrace = None
-        st_value = value.get("stackTrace") or value.get("stacktrace")
-        if st_value:
-            if isinstance(st_value, str):
-                stacktrace = st_value.split("\n")
-            else:
-                stacktrace = []
-                try:
-                    for frame in st_value:
-                        line = frame.get("lineNumber", "")
-                        file = frame.get("fileName", "&lt;anonymous&gt;")
-                        if line:
-                            file = f"{file}:{line}"
-                        meth = frame.get("methodName", "&lt;anonymous&gt;")
-                        if "className" in frame:
-                            meth = f"{frame['className']}.{meth}"
-                        msg = "    at %s (%s)"
-                        msg = msg % (meth, file)
-                        stacktrace.append(msg)
-                except TypeError:
-                    pass
-        if exception_class == UnexpectedAlertPresentException:
-            alert_text = None
-            if "data" in value:
-                alert_text = value["data"].get("text")
-            elif "alert" in value:
-                alert_text = value["alert"].get("text")
-            raise exception_class(message, screen, stacktrace, alert_text)
-&gt;       raise exception_class(message, screen, stacktrace)
-E       selenium.common.exceptions.WebDriverException: Message: Cannot start the 'com.kisanmitra.kisan_mitra' application. Consider checking the driver's troubleshooting documentation. Original error: 'com.kisanmitra.kisan_mitra.MainActivity' never started. Consider checking the driver's troubleshooting documentation.
+        error = value.get('error')
+        if not error:
+            return
+        message = value.get('message', error)
+        stacktrace = value.get('stacktrace', '')
+        # In theory, we should also be checking HTTP status codes.
+        # Java client, for example, prints a warning if the actual `error`
+        # value does not match to the response's HTTP status code.
+        exception_class: Type[sel_exceptions.WebDriverException] = ERROR_TO_EXC_MAPPING.get(
+            error, sel_exceptions.WebDriverException
+        )
+        if exception_class is sel_exceptions.WebDriverException and message:
+            if message == 'No such context found.':
+                exception_class = appium_exceptions.NoSuchContextException
+            elif message == 'That command could not be executed in the current context.':
+                exception_class = appium_exceptions.InvalidSwitchToTargetException
+        if exception_class is sel_exceptions.UnexpectedAlertPresentException:
+            raise sel_exceptions.UnexpectedAlertPresentException(
+                msg=message,
+                stacktrace=format_stacktrace(stacktrace),
+                alert_text=value.get('data'),
+            )
+&gt;       raise exception_class(msg=message, stacktrace=format_stacktrace(stacktrace))
+E       selenium.common.exceptions.WebDriverException: Message: io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10504ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work
 E       Stacktrace:
-E       UnknownError: Cannot start the 'com.kisanmitra.kisan_mitra' application. Consider checking the driver's troubleshooting documentation. Original error: 'com.kisanmitra.kisan_mitra.MainActivity' never started. Consider checking the driver's troubleshooting documentation.
-E           at getResponseForW3CError (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/node_modules/@appium/base-driver/build/lib/protocol/errors.js:846:36)
-E           at asyncHandler (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/node_modules/@appium/base-driver/build/lib/protocol/protocol.js:485:77)
-E           at process.processTicksAndRejections (node:internal/process/task_queues:95:5)
-E       The above error is caused by
-E       Error: Cannot start the 'com.kisanmitra.kisan_mitra' application. Consider checking the driver's troubleshooting documentation. Original error: 'com.kisanmitra.kisan_mitra.MainActivity' never started. Consider checking the driver's troubleshooting documentation.
-E           at ADB.startApp (/home/runner/.appium/node_modules/appium-uiautomator2-driver/node_modules/appium-adb/build/lib/tools/app-commands.js:612:15)
-E           at process.processTicksAndRejections (node:internal/process/task_queues:95:5)
-E           at async AndroidUiautomator2Driver.ensureAppStarts (/home/runner/.appium/node_modules/appium-uiautomator2-driver/build/lib/commands/aut.js:106:5)
-E           at async AndroidUiautomator2Driver.performPostExecSetup [as performSessionPostExecSetup] (/home/runner/.appium/node_modules/appium-uiautomator2-driver/build/lib/uiautomator2-server/session.js:202:9)
-E           at async AndroidUiautomator2Driver.startSession [as startUiAutomator2Session] (/home/runner/.appium/node_modules/appium-uiautomator2-driver/build/lib/uiautomator2-server/session.js:260:5)
-E           at async AndroidUiautomator2Driver.createSession (/home/runner/.appium/node_modules/appium-uiautomator2-driver/build/lib/driver.js:301:28)
-E           at async AppiumDriver.createSession (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/build/lib/appium.js:271:44)
-E           at async runCommandPromise (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/node_modules/@appium/base-driver/build/lib/basedriver/driver.js:119:24)
-E           at async AppiumDriver.executeCommand (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/node_modules/@appium/base-driver/build/lib/basedriver/driver.js:162:15)
-E           at async defaultBehavior (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/build/lib/appium.js:582:24)
-E           at async AppiumDriver.executeWrappedCommand (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/build/lib/appium.js:694:22)
-E           at async AppiumDriver.executeCommand (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/build/lib/appium.js:598:21)
-E           at async asyncHandler (/opt/hostedtoolcache/node/20.20.2/x64/lib/node_modules/appium/node_modules/@appium/base-driver/build/lib/protocol/protocol.js:401:25)
-/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/selenium/webdriver/remote/errorhandler.py:232: WebDriverException</t>
+E       io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10504ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work
+E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath1(AccessibilityNodeInfoDumper.java:306)
+E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodes(AccessibilityNodeInfoDumper.java:377)
+E       	at io.appium.uiautomator2.utils.ElementLocationHelpers.getXPathNodeMatch(ElementLocationHelpers.java:124)
+E       	at io.appium.uiautomator2.utils.ElementLocationHelpers.findElement(ElementLocationHelpers.java:151)
+E       	at io.appium.uiautomator2.handler.FindElement.safeHandle(FindElement.java:60)
+E       	at io.appium.uiautomator2.handler.request.SafeRequestHandler.handle(SafeRequestHandler.java:59)
+E       	at io.appium.uiautomator2.server.AppiumServlet.handleRequest(AppiumServlet.java:267)
+E       	at io.appium.uiautomator2.server.AppiumServlet.handleHttpRequest(AppiumServlet.java:261)
+E       	at io.appium.uiautomator2.http.ServerHandler.channelRead(ServerHandler.java:77)
+E       	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:357)
+E       	at io.netty.handler.codec.MessageToMessageDecoder.channelRead(MessageToMessageDecoder.java:107)
+E       	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:357)
+E       	at io.netty.channel.CombinedChannelDuplexHandler$DelegatingChannelHandlerContext.fireChannelRead(CombinedChannelDuplexHandler.java:434)
+E       	at io.netty.handler.codec.ByteToMessageDecoder.fireChannelRead(ByteToMessageDecoder.java:361)
+E       	at io.netty.handler.codec.ByteToMessageDecoder.channelRead(ByteToMessageDecoder.java:325)
+E       	at io.netty.channel.CombinedChannelDuplexHandler.channelRead(CombinedChannelDuplexHandler.java:249)
+E       	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:355)
+E       	at io.netty.handler.timeout.IdleStateHandler.channelRead(IdleStateHandler.java:288)
+E       	at io.netty.channel.AbstractChannelHandlerContext.fireChannelRead(AbstractChannelHandlerContext.java:355)
+E       	at io.netty.channel.DefaultChannelPipeline$HeadContext.channelRead(DefaultChannelPipeline.java:1429)
+E       	at io.netty.channel.DefaultChannelPipeline.fireChannelRead(DefaultChannelPipeline.java:918)
+E       	at io.netty.channel.nio.AbstractNioByteChannel$NioByteUnsafe.read(AbstractNioByteChannel.java:176)
+E       	at io.netty.channel.nio.AbstractNioChannel$AbstractNioUnsafe.handle(AbstractNioChannel.java:445)
+E       	at io.netty.channel.nio.NioIoHandler$DefaultNioRegistration.handle(NioIoHandler.java:388)
+E       	at io.netty.channel.nio.NioIoHandler.processSelectedKey(NioIoHandler.java:596)
+E       	at io.netty.channel.nio.NioIoHandler.processSelectedKeysOptimized(NioIoHandler.java:571)
+E       	at io.netty.channel.nio.NioIoHandler.processSelectedKeys(NioIoHandler.java:512)
+E       	at io.netty.channel.nio.NioIoHandler.run(NioIoHandler.java:484)
+E       	at io.netty.channel.SingleThreadIoEventLoop.runIo(SingleThreadIoEventLoop.java:225)
+E       	at io.netty.channel.SingleThreadIoEventLoop.run(SingleThreadIoEventLoop.java:196)
+E       	at io.netty.util.concurrent.SingleThreadEventExecutor$5.run(SingleThreadEventExecutor.java:1195)
+E       	at io.netty.util.internal.ThreadExecutorMap$2.run(ThreadExecutorMap.java:74)
+E       	at io.netty.util.concurrent.FastThreadLocalRunnable.run(FastThreadLocalRunnable.java:30)
+E       	at java.lang.Thread.run(Thread.java:919)
+E       Caused by: io.appium.uiautomator2.common.exceptions.UiAutomator2Exception: Timed out after 10504ms waiting for the root AccessibilityNodeInfo in the active window. Make sure the active window is not constantly hogging the main UI thread (e.g. the application is being idle long enough), so the accessibility manager could do its work
+E       	at io.appium.uiautomator2.utils.AXWindowHelpers.getActiveWindowRoot(AXWindowHelpers.java:107)
+E       	at io.appium.uiautomator2.utils.AXWindowHelpers.retrieveWindowRoots(AXWindowHelpers.java:87)
+E       	at io.appium.uiautomator2.utils.AXWindowHelpers.getCachedWindowRoots(AXWindowHelpers.java:68)
+E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.toStream(AccessibilityNodeInfoDumper.java:228)
+E       	at io.appium.uiautomator2.core.AccessibilityNodeInfoDumper.findNodesUsingXpath1(AccessibilityNodeInfoDumper.java:279)
+E       	... 33 more
+/opt/hostedtoolcache/Python/3.11.15/x64/lib/python3.11/site-packages/appium/webdriver/errorhandler.py:125: WebDriverException</t>
         </is>
       </c>
     </row>

</xml_diff>